<commit_message>
docs: author operational-metric-framework.md and synchronize provenance and tables
</commit_message>
<xml_diff>
--- a/results/manuscript_tables/thesis_tables.xlsx
+++ b/results/manuscript_tables/thesis_tables.xlsx
@@ -83,7 +83,7 @@
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Times New Roman"/>
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
@@ -5068,7 +5068,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="8.83203125" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13.5" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
@@ -5077,7 +5083,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2">
       <c r="A2" s="17" t="inlineStr">
         <is>
           <t>Baseline characteristic</t>
@@ -5131,7 +5137,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" ht="16" customHeight="1">
+    <row r="5">
       <c r="A5" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve"> Single</t>

</xml_diff>

<commit_message>
refactor: align chapters 1-5 with authoritative outlines, restore markdown tables, and excise hypothesis 2
</commit_message>
<xml_diff>
--- a/results/manuscript_tables/thesis_tables.xlsx
+++ b/results/manuscript_tables/thesis_tables.xlsx
@@ -1175,7 +1175,7 @@
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Hypothesis Testing (H1 &amp; H2)</t>
+          <t>Hypothesis Testing (H1)</t>
         </is>
       </c>
     </row>
@@ -3908,7 +3908,7 @@
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>Note. Master multi-pillar hypothesis evaluation matrix across Robustness, Resilience, and Generalizability. Demonstrates asymmetric trade-offs (H1) and confirms the values versus volatility paradigm (H2).</t>
+          <t>Note. Master multi-pillar hypothesis evaluation matrix across Robustness, Resilience, and Generalizability. Demonstrates asymmetric trade-offs (H1) and confirms the values versus volatility operational coupling.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: expand test suite to 48 tests, sanitize model tags, and standardize paths and styling
- Sanitize model naming checks in src/models/dual_track_eval.py, removing legacy internal tags (M0, M1*, M3) to strictly enforce Policy 3.2.
- Standardize TOP25_CLUSTERING_WB path import in src/etl/perform_top25_clustering.py from src.utils.paths.
- Adopt autofit_column_widths in src/analysis/season_analysis_volatility_runner.py from src.utils.excel_styling.
- Modernize src/utils/logger.py default logger name to 'final_thesis'.
- Enhance src/utils/excel_styling.py with comma-separated float parsing and APA table boundary helpers.
- Add comprehensive unit test suites in tests/test_panel_loader.py, tests/test_excel_styling.py, and tests/test_feature_pipeline.py (expanding test suite to 48 tests, 100% passing).
- Synchronize root README.md directory tree and update results/00_VERSION_CONTROL_AND_PROVENANCE.md to v4.45.
</commit_message>
<xml_diff>
--- a/results/manuscript_tables/thesis_tables.xlsx
+++ b/results/manuscript_tables/thesis_tables.xlsx
@@ -158,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -233,6 +233,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1547,7 +1550,7 @@
       <c r="I6" s="26" t="n">
         <v>192160</v>
       </c>
-      <c r="J6" s="30" t="inlineStr">
+      <c r="J6" s="31" t="inlineStr">
         <is>
           <t>+16.9%</t>
         </is>
@@ -1591,7 +1594,7 @@
       <c r="I7" s="26" t="n">
         <v>2738</v>
       </c>
-      <c r="J7" s="30" t="inlineStr">
+      <c r="J7" s="31" t="inlineStr">
         <is>
           <t>+32.3%</t>
         </is>
@@ -1613,17 +1616,17 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D8" s="30" t="inlineStr">
+      <c r="D8" s="31" t="inlineStr">
         <is>
           <t>1.63%</t>
         </is>
       </c>
-      <c r="E8" s="30" t="inlineStr">
+      <c r="E8" s="31" t="inlineStr">
         <is>
           <t>0.50%</t>
         </is>
       </c>
-      <c r="F8" s="30" t="inlineStr">
+      <c r="F8" s="31" t="inlineStr">
         <is>
           <t>1.47%</t>
         </is>
@@ -1638,12 +1641,12 @@
           <t>2.46% (LGA)</t>
         </is>
       </c>
-      <c r="I8" s="30" t="inlineStr">
+      <c r="I8" s="31" t="inlineStr">
         <is>
           <t>1.43%</t>
         </is>
       </c>
-      <c r="J8" s="30" t="inlineStr">
+      <c r="J8" s="31" t="inlineStr">
         <is>
           <t>+14.1%</t>
         </is>
@@ -1687,7 +1690,7 @@
       <c r="I9" s="29" t="n">
         <v>14.21</v>
       </c>
-      <c r="J9" s="30" t="inlineStr">
+      <c r="J9" s="31" t="inlineStr">
         <is>
           <t>+7.2%</t>
         </is>
@@ -1709,17 +1712,17 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D10" s="30" t="inlineStr">
+      <c r="D10" s="31" t="inlineStr">
         <is>
           <t>21.42%</t>
         </is>
       </c>
-      <c r="E10" s="30" t="inlineStr">
+      <c r="E10" s="31" t="inlineStr">
         <is>
           <t>3.30%</t>
         </is>
       </c>
-      <c r="F10" s="30" t="inlineStr">
+      <c r="F10" s="31" t="inlineStr">
         <is>
           <t>20.14%</t>
         </is>
@@ -1734,12 +1737,12 @@
           <t>28.07% (DFW)</t>
         </is>
       </c>
-      <c r="I10" s="30" t="inlineStr">
+      <c r="I10" s="31" t="inlineStr">
         <is>
           <t>20.31%</t>
         </is>
       </c>
-      <c r="J10" s="30" t="inlineStr">
+      <c r="J10" s="31" t="inlineStr">
         <is>
           <t>+5.5%</t>
         </is>
@@ -1783,7 +1786,7 @@
       <c r="I11" s="29" t="n">
         <v>19.69</v>
       </c>
-      <c r="J11" s="30" t="inlineStr">
+      <c r="J11" s="31" t="inlineStr">
         <is>
           <t>+4.5%</t>
         </is>
@@ -1827,7 +1830,7 @@
       <c r="I12" s="26" t="n">
         <v>68495531</v>
       </c>
-      <c r="J12" s="30" t="inlineStr">
+      <c r="J12" s="31" t="inlineStr">
         <is>
           <t>+3.9%</t>
         </is>
@@ -1871,7 +1874,7 @@
       <c r="I13" s="26" t="n">
         <v>51138</v>
       </c>
-      <c r="J13" s="30" t="inlineStr">
+      <c r="J13" s="31" t="inlineStr">
         <is>
           <t>+3.8%</t>
         </is>
@@ -1915,7 +1918,7 @@
       <c r="I14" s="29" t="n">
         <v>540.34</v>
       </c>
-      <c r="J14" s="30" t="inlineStr">
+      <c r="J14" s="31" t="inlineStr">
         <is>
           <t>-22.5%</t>
         </is>
@@ -1959,7 +1962,7 @@
       <c r="I15" s="26" t="n">
         <v>2784</v>
       </c>
-      <c r="J15" s="30" t="inlineStr">
+      <c r="J15" s="31" t="inlineStr">
         <is>
           <t>-4.0%</t>
         </is>
@@ -1981,13 +1984,13 @@
           <t>ratio</t>
         </is>
       </c>
-      <c r="D16" s="35" t="n">
+      <c r="D16" s="36" t="n">
         <v>0.8728</v>
       </c>
-      <c r="E16" s="35" t="n">
+      <c r="E16" s="36" t="n">
         <v>0.2</v>
       </c>
-      <c r="F16" s="35" t="n">
+      <c r="F16" s="36" t="n">
         <v>0.9064</v>
       </c>
       <c r="G16" s="9" t="inlineStr">
@@ -2000,10 +2003,10 @@
           <t>1.1240 (LGA)</t>
         </is>
       </c>
-      <c r="I16" s="35" t="n">
+      <c r="I16" s="36" t="n">
         <v>0.825</v>
       </c>
-      <c r="J16" s="30" t="inlineStr">
+      <c r="J16" s="31" t="inlineStr">
         <is>
           <t>+5.8%</t>
         </is>
@@ -2025,17 +2028,17 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D17" s="30" t="inlineStr">
+      <c r="D17" s="31" t="inlineStr">
         <is>
           <t>47.45%</t>
         </is>
       </c>
-      <c r="E17" s="30" t="inlineStr">
+      <c r="E17" s="31" t="inlineStr">
         <is>
           <t>10.98%</t>
         </is>
       </c>
-      <c r="F17" s="30" t="inlineStr">
+      <c r="F17" s="31" t="inlineStr">
         <is>
           <t>44.41%</t>
         </is>
@@ -2050,12 +2053,12 @@
           <t>66.32% (DFW)</t>
         </is>
       </c>
-      <c r="I17" s="30" t="inlineStr">
+      <c r="I17" s="31" t="inlineStr">
         <is>
           <t>51.39%</t>
         </is>
       </c>
-      <c r="J17" s="30" t="inlineStr">
+      <c r="J17" s="31" t="inlineStr">
         <is>
           <t>-7.7%</t>
         </is>
@@ -2077,17 +2080,17 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D18" s="30" t="inlineStr">
+      <c r="D18" s="31" t="inlineStr">
         <is>
           <t>52.55%</t>
         </is>
       </c>
-      <c r="E18" s="30" t="inlineStr">
+      <c r="E18" s="31" t="inlineStr">
         <is>
           <t>10.98%</t>
         </is>
       </c>
-      <c r="F18" s="30" t="inlineStr">
+      <c r="F18" s="31" t="inlineStr">
         <is>
           <t>55.59%</t>
         </is>
@@ -2102,12 +2105,12 @@
           <t>66.42% (EWR)</t>
         </is>
       </c>
-      <c r="I18" s="30" t="inlineStr">
+      <c r="I18" s="31" t="inlineStr">
         <is>
           <t>48.61%</t>
         </is>
       </c>
-      <c r="J18" s="30" t="inlineStr">
+      <c r="J18" s="31" t="inlineStr">
         <is>
           <t>+8.1%</t>
         </is>
@@ -2151,7 +2154,7 @@
       <c r="I19" s="26" t="n">
         <v>13103484</v>
       </c>
-      <c r="J19" s="30" t="inlineStr">
+      <c r="J19" s="31" t="inlineStr">
         <is>
           <t>+25.0%</t>
         </is>
@@ -2195,7 +2198,7 @@
       <c r="I20" s="29" t="n">
         <v>171.1</v>
       </c>
-      <c r="J20" s="30" t="inlineStr">
+      <c r="J20" s="31" t="inlineStr">
         <is>
           <t>-1.6%</t>
         </is>
@@ -2217,17 +2220,17 @@
           <t>%</t>
         </is>
       </c>
-      <c r="D21" s="31" t="inlineStr">
+      <c r="D21" s="32" t="inlineStr">
         <is>
           <t>85.08%</t>
         </is>
       </c>
-      <c r="E21" s="31" t="inlineStr">
+      <c r="E21" s="32" t="inlineStr">
         <is>
           <t>0.82%</t>
         </is>
       </c>
-      <c r="F21" s="31" t="inlineStr">
+      <c r="F21" s="32" t="inlineStr">
         <is>
           <t>85.26%</t>
         </is>
@@ -2242,12 +2245,12 @@
           <t>86.12% (EWR)</t>
         </is>
       </c>
-      <c r="I21" s="31" t="inlineStr">
+      <c r="I21" s="32" t="inlineStr">
         <is>
           <t>84.73%</t>
         </is>
       </c>
-      <c r="J21" s="31" t="inlineStr">
+      <c r="J21" s="32" t="inlineStr">
         <is>
           <t>+0.4%</t>
         </is>
@@ -2780,7 +2783,7 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="K14" s="34" t="n">
+      <c r="K14" s="35" t="n">
         <v>1.23</v>
       </c>
       <c r="L14" s="13" t="inlineStr">
@@ -2875,10 +2878,10 @@
           <t>Lag t-1 (1 hr post-departure)</t>
         </is>
       </c>
-      <c r="B6" s="35" t="n">
+      <c r="B6" s="36" t="n">
         <v>0.1987</v>
       </c>
-      <c r="C6" s="30" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>3.95%</t>
         </is>
@@ -2898,10 +2901,10 @@
           <t>Same-Hour Departure t (Gate departure)</t>
         </is>
       </c>
-      <c r="B7" s="35" t="n">
+      <c r="B7" s="36" t="n">
         <v>0.3403</v>
       </c>
-      <c r="C7" s="30" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
         <is>
           <t>11.58%</t>
         </is>
@@ -2921,10 +2924,10 @@
           <t>Lead t+1 (1 hr pre-departure)</t>
         </is>
       </c>
-      <c r="B8" s="35" t="n">
+      <c r="B8" s="36" t="n">
         <v>0.4913</v>
       </c>
-      <c r="C8" s="30" t="inlineStr">
+      <c r="C8" s="31" t="inlineStr">
         <is>
           <t>24.13%</t>
         </is>
@@ -2944,10 +2947,10 @@
           <t>Lead t+2 (2 hr pre-departure)</t>
         </is>
       </c>
-      <c r="B9" s="35" t="n">
+      <c r="B9" s="36" t="n">
         <v>0.4876</v>
       </c>
-      <c r="C9" s="30" t="inlineStr">
+      <c r="C9" s="31" t="inlineStr">
         <is>
           <t>23.78%</t>
         </is>
@@ -2967,10 +2970,10 @@
           <t>Lead t+3 (3 hr pre-departure)</t>
         </is>
       </c>
-      <c r="B10" s="35" t="n">
+      <c r="B10" s="36" t="n">
         <v>0.38</v>
       </c>
-      <c r="C10" s="30" t="inlineStr">
+      <c r="C10" s="31" t="inlineStr">
         <is>
           <t>14.44%</t>
         </is>
@@ -2990,10 +2993,10 @@
           <t>Convolved Passenger Show-Up Curve</t>
         </is>
       </c>
-      <c r="B11" s="35" t="n">
+      <c r="B11" s="36" t="n">
         <v>0.6985</v>
       </c>
-      <c r="C11" s="30" t="inlineStr">
+      <c r="C11" s="31" t="inlineStr">
         <is>
           <t>48.78%</t>
         </is>
@@ -3013,15 +3016,15 @@
           <t>Show-Up Curve x T-100 Load Factor</t>
         </is>
       </c>
-      <c r="B12" s="36" t="n">
+      <c r="B12" s="37" t="n">
         <v>0.7060999999999999</v>
       </c>
-      <c r="C12" s="31" t="inlineStr">
+      <c r="C12" s="32" t="inlineStr">
         <is>
           <t>49.85%</t>
         </is>
       </c>
-      <c r="D12" s="34" t="n">
+      <c r="D12" s="35" t="n">
         <v>90.56</v>
       </c>
       <c r="E12" s="13" t="inlineStr">
@@ -3156,22 +3159,22 @@
           <t>Daily Persistence Benchmark (y_t-24)</t>
         </is>
       </c>
-      <c r="D6" s="35" t="n">
+      <c r="D6" s="36" t="n">
         <v>0.4412</v>
       </c>
-      <c r="E6" s="35" t="n">
+      <c r="E6" s="36" t="n">
         <v>0.6719000000000001</v>
       </c>
-      <c r="F6" s="37" t="n">
+      <c r="F6" s="38" t="n">
         <v>253.6</v>
       </c>
-      <c r="G6" s="37" t="n">
+      <c r="G6" s="38" t="n">
         <v>179.3</v>
       </c>
-      <c r="H6" s="32" t="n">
+      <c r="H6" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="I6" s="37" t="n">
+      <c r="I6" s="38" t="n">
         <v>-0.7</v>
       </c>
       <c r="J6" s="9" t="inlineStr">
@@ -3196,22 +3199,22 @@
           <t>Deterministic Flight Schedule Model (convolved show-up curve)</t>
         </is>
       </c>
-      <c r="D7" s="35" t="n">
+      <c r="D7" s="36" t="n">
         <v>0.4912</v>
       </c>
-      <c r="E7" s="35" t="n">
+      <c r="E7" s="36" t="n">
         <v>0.498</v>
       </c>
-      <c r="F7" s="37" t="n">
+      <c r="F7" s="38" t="n">
         <v>313.4</v>
       </c>
-      <c r="G7" s="37" t="n">
+      <c r="G7" s="38" t="n">
         <v>215.9</v>
       </c>
-      <c r="H7" s="32" t="n">
+      <c r="H7" s="33" t="n">
         <v>0.945</v>
       </c>
-      <c r="I7" s="37" t="n">
+      <c r="I7" s="38" t="n">
         <v>-42.1</v>
       </c>
       <c r="J7" s="9" t="inlineStr">
@@ -3236,22 +3239,22 @@
           <t>Supervised Machine Learning Model (Decision Trees &amp; OTP)</t>
         </is>
       </c>
-      <c r="D8" s="35" t="n">
+      <c r="D8" s="36" t="n">
         <v>0.5455</v>
       </c>
-      <c r="E8" s="35" t="n">
+      <c r="E8" s="36" t="n">
         <v>0.6178</v>
       </c>
-      <c r="F8" s="37" t="n">
+      <c r="F8" s="38" t="n">
         <v>273.5</v>
       </c>
-      <c r="G8" s="37" t="n">
+      <c r="G8" s="38" t="n">
         <v>178</v>
       </c>
-      <c r="H8" s="32" t="n">
+      <c r="H8" s="33" t="n">
         <v>0.779</v>
       </c>
-      <c r="I8" s="37" t="n">
+      <c r="I8" s="38" t="n">
         <v>-18.4</v>
       </c>
       <c r="J8" s="9" t="inlineStr">
@@ -3276,22 +3279,22 @@
           <t>Dynamic Two-Stage Hybrid Model (Schedule + Real-time feedback)</t>
         </is>
       </c>
-      <c r="D9" s="36" t="n">
+      <c r="D9" s="37" t="n">
         <v>0.712</v>
       </c>
-      <c r="E9" s="36" t="n">
+      <c r="E9" s="37" t="n">
         <v>0.7483</v>
       </c>
-      <c r="F9" s="38" t="n">
+      <c r="F9" s="39" t="n">
         <v>222.1</v>
       </c>
-      <c r="G9" s="38" t="n">
+      <c r="G9" s="39" t="n">
         <v>142.8</v>
       </c>
-      <c r="H9" s="33" t="n">
+      <c r="H9" s="34" t="n">
         <v>0.662</v>
       </c>
-      <c r="I9" s="38" t="n">
+      <c r="I9" s="39" t="n">
         <v>-8.5</v>
       </c>
       <c r="J9" s="13" t="inlineStr">
@@ -3472,10 +3475,10 @@
           <t>MASE &lt; 0.700</t>
         </is>
       </c>
-      <c r="E7" s="32" t="n">
+      <c r="E7" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="32" t="n">
+      <c r="F7" s="33" t="n">
         <v>0.945</v>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -3483,7 +3486,7 @@
           <t>0.680--0.700</t>
         </is>
       </c>
-      <c r="H7" s="32" t="n">
+      <c r="H7" s="33" t="n">
         <v>0.662</v>
       </c>
       <c r="I7" s="9" t="inlineStr">
@@ -3607,13 +3610,13 @@
           <t>Lowest Shock MASE</t>
         </is>
       </c>
-      <c r="E10" s="32" t="n">
+      <c r="E10" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="32" t="n">
+      <c r="F10" s="33" t="n">
         <v>1.082</v>
       </c>
-      <c r="G10" s="32" t="n">
+      <c r="G10" s="33" t="n">
         <v>0.8120000000000001</v>
       </c>
       <c r="H10" s="9" t="inlineStr">
@@ -3832,7 +3835,7 @@
           <t>Minimal Penalty (&lt;= 10%)</t>
         </is>
       </c>
-      <c r="E15" s="30" t="inlineStr">
+      <c r="E15" s="31" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
@@ -3879,7 +3882,7 @@
           <t>DeltaMASE &lt;= 10.0%</t>
         </is>
       </c>
-      <c r="E16" s="31" t="inlineStr">
+      <c r="E16" s="32" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
@@ -4019,10 +4022,10 @@
           <t>Daily Persistence Benchmark (y_t-24)</t>
         </is>
       </c>
-      <c r="D6" s="37" t="n">
+      <c r="D6" s="38" t="n">
         <v>253.6</v>
       </c>
-      <c r="E6" s="32" t="n">
+      <c r="E6" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -4057,10 +4060,10 @@
           <t>Deterministic Flight Schedule Model</t>
         </is>
       </c>
-      <c r="D7" s="37" t="n">
+      <c r="D7" s="38" t="n">
         <v>313.4</v>
       </c>
-      <c r="E7" s="32" t="n">
+      <c r="E7" s="33" t="n">
         <v>0.945</v>
       </c>
       <c r="F7" s="9" t="inlineStr">
@@ -4095,7 +4098,7 @@
           <t>Supervised Machine Learning Model</t>
         </is>
       </c>
-      <c r="D8" s="37" t="n">
+      <c r="D8" s="38" t="n">
         <v>273.5</v>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -4135,10 +4138,10 @@
           <t>Dynamic Two-Stage Hybrid Model</t>
         </is>
       </c>
-      <c r="D9" s="38" t="n">
+      <c r="D9" s="39" t="n">
         <v>222.1</v>
       </c>
-      <c r="E9" s="33" t="n">
+      <c r="E9" s="34" t="n">
         <v>0.662</v>
       </c>
       <c r="F9" s="13" t="inlineStr">
@@ -4277,10 +4280,10 @@
           <t>Daily Persistence Benchmark (y_t-24)</t>
         </is>
       </c>
-      <c r="D6" s="37" t="n">
+      <c r="D6" s="38" t="n">
         <v>398.2</v>
       </c>
-      <c r="E6" s="32" t="n">
+      <c r="E6" s="33" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="29" t="n">
@@ -4318,10 +4321,10 @@
           <t>Deterministic Flight Schedule Model</t>
         </is>
       </c>
-      <c r="D7" s="37" t="n">
+      <c r="D7" s="38" t="n">
         <v>412.8</v>
       </c>
-      <c r="E7" s="32" t="n">
+      <c r="E7" s="33" t="n">
         <v>1.082</v>
       </c>
       <c r="F7" s="29" t="n">
@@ -4359,10 +4362,10 @@
           <t>Supervised Machine Learning Model</t>
         </is>
       </c>
-      <c r="D8" s="37" t="n">
+      <c r="D8" s="38" t="n">
         <v>318.4</v>
       </c>
-      <c r="E8" s="32" t="n">
+      <c r="E8" s="33" t="n">
         <v>0.8120000000000001</v>
       </c>
       <c r="F8" s="29" t="n">
@@ -4400,13 +4403,13 @@
           <t>Dynamic Two-Stage Hybrid Model</t>
         </is>
       </c>
-      <c r="D9" s="38" t="n">
+      <c r="D9" s="39" t="n">
         <v>254.2</v>
       </c>
-      <c r="E9" s="33" t="n">
+      <c r="E9" s="34" t="n">
         <v>0.694</v>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="35" t="n">
         <v>1.05</v>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -4545,21 +4548,21 @@
           <t>Daily Persistence Benchmark (y_t-24)</t>
         </is>
       </c>
-      <c r="D6" s="37" t="n">
+      <c r="D6" s="38" t="n">
         <v>253.6</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="E6" s="38" t="n">
         <v>253.6</v>
       </c>
       <c r="F6" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="30" t="inlineStr">
+      <c r="G6" s="31" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="H6" s="30" t="inlineStr">
+      <c r="H6" s="31" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
@@ -4586,16 +4589,16 @@
           <t>Deterministic Flight Schedule Model</t>
         </is>
       </c>
-      <c r="D7" s="37" t="n">
+      <c r="D7" s="38" t="n">
         <v>313.4</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="E7" s="38" t="n">
         <v>326.5</v>
       </c>
       <c r="F7" s="29" t="n">
         <v>1.04</v>
       </c>
-      <c r="G7" s="30" t="inlineStr">
+      <c r="G7" s="31" t="inlineStr">
         <is>
           <t>+4.2%</t>
         </is>
@@ -4627,16 +4630,16 @@
           <t>Supervised Machine Learning Model</t>
         </is>
       </c>
-      <c r="D8" s="37" t="n">
+      <c r="D8" s="38" t="n">
         <v>273.5</v>
       </c>
-      <c r="E8" s="37" t="n">
+      <c r="E8" s="38" t="n">
         <v>295.1</v>
       </c>
       <c r="F8" s="29" t="n">
         <v>1.08</v>
       </c>
-      <c r="G8" s="30" t="inlineStr">
+      <c r="G8" s="31" t="inlineStr">
         <is>
           <t>+7.9%</t>
         </is>
@@ -4668,16 +4671,16 @@
           <t>Dynamic Two-Stage Hybrid Model</t>
         </is>
       </c>
-      <c r="D9" s="38" t="n">
+      <c r="D9" s="39" t="n">
         <v>222.1</v>
       </c>
-      <c r="E9" s="38" t="n">
+      <c r="E9" s="39" t="n">
         <v>264.3</v>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="35" t="n">
         <v>1.19</v>
       </c>
-      <c r="G9" s="31" t="inlineStr">
+      <c r="G9" s="32" t="inlineStr">
         <is>
           <t>+19.0%</t>
         </is>
@@ -5581,18 +5584,14 @@
       <c r="H6" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="9" t="inlineStr">
-        <is>
-          <t>5,336.00</t>
-        </is>
+      <c r="I6" s="30" t="n">
+        <v>5336</v>
       </c>
       <c r="J6" s="29" t="n">
         <v>10</v>
       </c>
-      <c r="K6" s="9" t="inlineStr">
-        <is>
-          <t>1,316.00</t>
-        </is>
+      <c r="K6" s="30" t="n">
+        <v>1316</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -5624,10 +5623,8 @@
       <c r="H7" s="29" t="n">
         <v>-105</v>
       </c>
-      <c r="I7" s="9" t="inlineStr">
-        <is>
-          <t>3,695.00</t>
-        </is>
+      <c r="I7" s="30" t="n">
+        <v>3695</v>
       </c>
       <c r="J7" s="29" t="n">
         <v>-10</v>
@@ -5650,42 +5647,42 @@
       <c r="C8" s="26" t="n">
         <v>13153654</v>
       </c>
-      <c r="D8" s="30" t="inlineStr">
+      <c r="D8" s="31" t="inlineStr">
         <is>
           <t>20.12%</t>
         </is>
       </c>
-      <c r="E8" s="30" t="inlineStr">
+      <c r="E8" s="31" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="F8" s="30" t="inlineStr">
+      <c r="F8" s="31" t="inlineStr">
         <is>
           <t>40.09%</t>
         </is>
       </c>
-      <c r="G8" s="30" t="inlineStr">
+      <c r="G8" s="31" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="H8" s="30" t="inlineStr">
+      <c r="H8" s="31" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I8" s="30" t="inlineStr">
+      <c r="I8" s="31" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>
       </c>
-      <c r="J8" s="30" t="inlineStr">
+      <c r="J8" s="31" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="K8" s="30" t="inlineStr">
+      <c r="K8" s="31" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>
@@ -5705,42 +5702,42 @@
       <c r="C9" s="26" t="n">
         <v>13153654</v>
       </c>
-      <c r="D9" s="30" t="inlineStr">
+      <c r="D9" s="31" t="inlineStr">
         <is>
           <t>2.03%</t>
         </is>
       </c>
-      <c r="E9" s="30" t="inlineStr">
+      <c r="E9" s="31" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="F9" s="30" t="inlineStr">
+      <c r="F9" s="31" t="inlineStr">
         <is>
           <t>14.09%</t>
         </is>
       </c>
-      <c r="G9" s="30" t="inlineStr">
+      <c r="G9" s="31" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="H9" s="30" t="inlineStr">
+      <c r="H9" s="31" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I9" s="30" t="inlineStr">
+      <c r="I9" s="31" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>
       </c>
-      <c r="J9" s="30" t="inlineStr">
+      <c r="J9" s="31" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="K9" s="30" t="inlineStr">
+      <c r="K9" s="31" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>
@@ -5838,10 +5835,8 @@
       <c r="C12" s="26" t="n">
         <v>13153654</v>
       </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>1,052.12</t>
-        </is>
+      <c r="D12" s="30" t="n">
+        <v>1052.12</v>
       </c>
       <c r="E12" s="29" t="n">
         <v>867</v>
@@ -5855,18 +5850,14 @@
       <c r="H12" s="29" t="n">
         <v>67</v>
       </c>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>5,095.00</t>
-        </is>
+      <c r="I12" s="30" t="n">
+        <v>5095</v>
       </c>
       <c r="J12" s="29" t="n">
         <v>230</v>
       </c>
-      <c r="K12" s="9" t="inlineStr">
-        <is>
-          <t>2,550.00</t>
-        </is>
+      <c r="K12" s="30" t="n">
+        <v>2550</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -5883,41 +5874,29 @@
       <c r="C13" s="26" t="n">
         <v>422096</v>
       </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>4,962.40</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>2,512.00</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>7,019.66</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>5,480.00</t>
-        </is>
+      <c r="D13" s="30" t="n">
+        <v>4962.4</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <v>2512</v>
+      </c>
+      <c r="F13" s="30" t="n">
+        <v>7019.66</v>
+      </c>
+      <c r="G13" s="30" t="n">
+        <v>5480</v>
       </c>
       <c r="H13" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="I13" s="9" t="inlineStr">
-        <is>
-          <t>145,200.00</t>
-        </is>
+      <c r="I13" s="30" t="n">
+        <v>145200</v>
       </c>
       <c r="J13" s="29" t="n">
         <v>120</v>
       </c>
-      <c r="K13" s="9" t="inlineStr">
-        <is>
-          <t>19,200.00</t>
-        </is>
+      <c r="K13" s="30" t="n">
+        <v>19200</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -5934,41 +5913,29 @@
       <c r="C14" s="26" t="n">
         <v>422096</v>
       </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>4,030.05</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>1,927.00</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>5,938.42</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>4,380.00</t>
-        </is>
+      <c r="D14" s="30" t="n">
+        <v>4030.05</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <v>1927</v>
+      </c>
+      <c r="F14" s="30" t="n">
+        <v>5938.42</v>
+      </c>
+      <c r="G14" s="30" t="n">
+        <v>4380</v>
       </c>
       <c r="H14" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="9" t="inlineStr">
-        <is>
-          <t>128,500.00</t>
-        </is>
+      <c r="I14" s="30" t="n">
+        <v>128500</v>
       </c>
       <c r="J14" s="29" t="n">
         <v>85</v>
       </c>
-      <c r="K14" s="9" t="inlineStr">
-        <is>
-          <t>15,800.00</t>
-        </is>
+      <c r="K14" s="30" t="n">
+        <v>15800</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -5985,42 +5952,42 @@
       <c r="C15" s="26" t="n">
         <v>422096</v>
       </c>
-      <c r="D15" s="30" t="inlineStr">
+      <c r="D15" s="31" t="inlineStr">
         <is>
           <t>81.21%</t>
         </is>
       </c>
-      <c r="E15" s="30" t="inlineStr">
+      <c r="E15" s="31" t="inlineStr">
         <is>
           <t>83.40%</t>
         </is>
       </c>
-      <c r="F15" s="30" t="inlineStr">
+      <c r="F15" s="31" t="inlineStr">
         <is>
           <t>11.80%</t>
         </is>
       </c>
-      <c r="G15" s="30" t="inlineStr">
+      <c r="G15" s="31" t="inlineStr">
         <is>
           <t>12.50%</t>
         </is>
       </c>
-      <c r="H15" s="30" t="inlineStr">
+      <c r="H15" s="31" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I15" s="30" t="inlineStr">
+      <c r="I15" s="31" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>
       </c>
-      <c r="J15" s="30" t="inlineStr">
+      <c r="J15" s="31" t="inlineStr">
         <is>
           <t>58.40%</t>
         </is>
       </c>
-      <c r="K15" s="30" t="inlineStr">
+      <c r="K15" s="31" t="inlineStr">
         <is>
           <t>94.20%</t>
         </is>
@@ -6040,42 +6007,42 @@
       <c r="C16" s="27" t="n">
         <v>22051557</v>
       </c>
-      <c r="D16" s="31" t="inlineStr">
+      <c r="D16" s="32" t="inlineStr">
         <is>
           <t>51.39%</t>
         </is>
       </c>
-      <c r="E16" s="31" t="inlineStr">
+      <c r="E16" s="32" t="inlineStr">
         <is>
           <t>50.73%</t>
         </is>
       </c>
-      <c r="F16" s="31" t="inlineStr">
+      <c r="F16" s="32" t="inlineStr">
         <is>
           <t>11.74%</t>
         </is>
       </c>
-      <c r="G16" s="31" t="inlineStr">
+      <c r="G16" s="32" t="inlineStr">
         <is>
           <t>16.20%</t>
         </is>
       </c>
-      <c r="H16" s="31" t="inlineStr">
+      <c r="H16" s="32" t="inlineStr">
         <is>
           <t>33.58%</t>
         </is>
       </c>
-      <c r="I16" s="31" t="inlineStr">
+      <c r="I16" s="32" t="inlineStr">
         <is>
           <t>76.04%</t>
         </is>
       </c>
-      <c r="J16" s="31" t="inlineStr">
+      <c r="J16" s="32" t="inlineStr">
         <is>
           <t>35.69%</t>
         </is>
       </c>
-      <c r="K16" s="31" t="inlineStr">
+      <c r="K16" s="32" t="inlineStr">
         <is>
           <t>70.09%</t>
         </is>
@@ -6415,7 +6382,7 @@
       <c r="C6" s="26" t="n">
         <v>500</v>
       </c>
-      <c r="D6" s="30" t="inlineStr">
+      <c r="D6" s="31" t="inlineStr">
         <is>
           <t>37.3%</t>
         </is>
@@ -6423,7 +6390,7 @@
       <c r="E6" s="26" t="n">
         <v>1123386</v>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="F6" s="33" t="n">
         <v>0.605</v>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -6439,12 +6406,12 @@
           <t>9.85 min</t>
         </is>
       </c>
-      <c r="J6" s="30" t="inlineStr">
+      <c r="J6" s="31" t="inlineStr">
         <is>
           <t>18.00%</t>
         </is>
       </c>
-      <c r="K6" s="30" t="inlineStr">
+      <c r="K6" s="31" t="inlineStr">
         <is>
           <t>0.89%</t>
         </is>
@@ -6464,7 +6431,7 @@
       <c r="C7" s="26" t="n">
         <v>426</v>
       </c>
-      <c r="D7" s="30" t="inlineStr">
+      <c r="D7" s="31" t="inlineStr">
         <is>
           <t>31.8%</t>
         </is>
@@ -6472,7 +6439,7 @@
       <c r="E7" s="26" t="n">
         <v>1187095</v>
       </c>
-      <c r="F7" s="32" t="n">
+      <c r="F7" s="33" t="n">
         <v>0.589</v>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -6488,12 +6455,12 @@
           <t>15.14 min</t>
         </is>
       </c>
-      <c r="J7" s="30" t="inlineStr">
+      <c r="J7" s="31" t="inlineStr">
         <is>
           <t>23.23%</t>
         </is>
       </c>
-      <c r="K7" s="30" t="inlineStr">
+      <c r="K7" s="31" t="inlineStr">
         <is>
           <t>1.36%</t>
         </is>
@@ -6513,7 +6480,7 @@
       <c r="C8" s="26" t="n">
         <v>224</v>
       </c>
-      <c r="D8" s="30" t="inlineStr">
+      <c r="D8" s="31" t="inlineStr">
         <is>
           <t>16.7%</t>
         </is>
@@ -6521,7 +6488,7 @@
       <c r="E8" s="26" t="n">
         <v>1305968</v>
       </c>
-      <c r="F8" s="32" t="n">
+      <c r="F8" s="33" t="n">
         <v>0.576</v>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -6537,12 +6504,12 @@
           <t>24.17 min</t>
         </is>
       </c>
-      <c r="J8" s="30" t="inlineStr">
+      <c r="J8" s="31" t="inlineStr">
         <is>
           <t>31.04%</t>
         </is>
       </c>
-      <c r="K8" s="30" t="inlineStr">
+      <c r="K8" s="31" t="inlineStr">
         <is>
           <t>3.16%</t>
         </is>
@@ -6562,7 +6529,7 @@
       <c r="C9" s="27" t="n">
         <v>191</v>
       </c>
-      <c r="D9" s="31" t="inlineStr">
+      <c r="D9" s="32" t="inlineStr">
         <is>
           <t>14.2%</t>
         </is>
@@ -6570,7 +6537,7 @@
       <c r="E9" s="27" t="n">
         <v>1215636</v>
       </c>
-      <c r="F9" s="33" t="n">
+      <c r="F9" s="34" t="n">
         <v>0.597</v>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -6578,7 +6545,7 @@
           <t>55.78 min</t>
         </is>
       </c>
-      <c r="H9" s="34" t="n">
+      <c r="H9" s="35" t="n">
         <v>33.07</v>
       </c>
       <c r="I9" s="13" t="inlineStr">
@@ -6586,12 +6553,12 @@
           <t>16.51 min</t>
         </is>
       </c>
-      <c r="J9" s="31" t="inlineStr">
+      <c r="J9" s="32" t="inlineStr">
         <is>
           <t>24.33%</t>
         </is>
       </c>
-      <c r="K9" s="31" t="inlineStr">
+      <c r="K9" s="32" t="inlineStr">
         <is>
           <t>1.82%</t>
         </is>
@@ -6727,7 +6694,7 @@
       <c r="E6" s="26" t="n">
         <v>1246150</v>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="F6" s="33" t="n">
         <v>0.604</v>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -6743,7 +6710,7 @@
           <t>15.78 min</t>
         </is>
       </c>
-      <c r="J6" s="30" t="inlineStr">
+      <c r="J6" s="31" t="inlineStr">
         <is>
           <t>23.54%</t>
         </is>
@@ -6769,7 +6736,7 @@
       <c r="E7" s="26" t="n">
         <v>1076625</v>
       </c>
-      <c r="F7" s="32" t="n">
+      <c r="F7" s="33" t="n">
         <v>0.601</v>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -6785,7 +6752,7 @@
           <t>11.69 min</t>
         </is>
       </c>
-      <c r="J7" s="30" t="inlineStr">
+      <c r="J7" s="31" t="inlineStr">
         <is>
           <t>19.44%</t>
         </is>
@@ -6811,7 +6778,7 @@
       <c r="E8" s="26" t="n">
         <v>1123368</v>
       </c>
-      <c r="F8" s="32" t="n">
+      <c r="F8" s="33" t="n">
         <v>0.594</v>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -6827,7 +6794,7 @@
           <t>12.22 min</t>
         </is>
       </c>
-      <c r="J8" s="30" t="inlineStr">
+      <c r="J8" s="31" t="inlineStr">
         <is>
           <t>20.05%</t>
         </is>
@@ -6853,7 +6820,7 @@
       <c r="E9" s="26" t="n">
         <v>1254744</v>
       </c>
-      <c r="F9" s="32" t="n">
+      <c r="F9" s="33" t="n">
         <v>0.589</v>
       </c>
       <c r="G9" s="9" t="inlineStr">
@@ -6869,7 +6836,7 @@
           <t>15.39 min</t>
         </is>
       </c>
-      <c r="J9" s="30" t="inlineStr">
+      <c r="J9" s="31" t="inlineStr">
         <is>
           <t>23.35%</t>
         </is>
@@ -6895,7 +6862,7 @@
       <c r="E10" s="26" t="n">
         <v>1241359</v>
       </c>
-      <c r="F10" s="32" t="n">
+      <c r="F10" s="33" t="n">
         <v>0.592</v>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -6911,7 +6878,7 @@
           <t>16.61 min</t>
         </is>
       </c>
-      <c r="J10" s="30" t="inlineStr">
+      <c r="J10" s="31" t="inlineStr">
         <is>
           <t>24.76%</t>
         </is>
@@ -6937,7 +6904,7 @@
       <c r="E11" s="26" t="n">
         <v>1089699</v>
       </c>
-      <c r="F11" s="32" t="n">
+      <c r="F11" s="33" t="n">
         <v>0.602</v>
       </c>
       <c r="G11" s="9" t="inlineStr">
@@ -6953,7 +6920,7 @@
           <t>14.64 min</t>
         </is>
       </c>
-      <c r="J11" s="30" t="inlineStr">
+      <c r="J11" s="31" t="inlineStr">
         <is>
           <t>22.47%</t>
         </is>
@@ -6979,7 +6946,7 @@
       <c r="E12" s="27" t="n">
         <v>1279017</v>
       </c>
-      <c r="F12" s="33" t="n">
+      <c r="F12" s="34" t="n">
         <v>0.577</v>
       </c>
       <c r="G12" s="13" t="inlineStr">
@@ -6987,7 +6954,7 @@
           <t>58.07 min</t>
         </is>
       </c>
-      <c r="H12" s="34" t="n">
+      <c r="H12" s="35" t="n">
         <v>33.4</v>
       </c>
       <c r="I12" s="13" t="inlineStr">
@@ -6995,7 +6962,7 @@
           <t>17.78 min</t>
         </is>
       </c>
-      <c r="J12" s="31" t="inlineStr">
+      <c r="J12" s="32" t="inlineStr">
         <is>
           <t>25.60%</t>
         </is>
@@ -7126,10 +7093,10 @@
           <t>Top 25 Airfields</t>
         </is>
       </c>
-      <c r="E6" s="35" t="n">
+      <c r="E6" s="36" t="n">
         <v>0.4572</v>
       </c>
-      <c r="F6" s="30" t="inlineStr">
+      <c r="F6" s="31" t="inlineStr">
         <is>
           <t>20.90%</t>
         </is>
@@ -7169,10 +7136,10 @@
           <t>Top 25 Airfields</t>
         </is>
       </c>
-      <c r="E7" s="35" t="n">
+      <c r="E7" s="36" t="n">
         <v>0.6704</v>
       </c>
-      <c r="F7" s="30" t="inlineStr">
+      <c r="F7" s="31" t="inlineStr">
         <is>
           <t>44.94%</t>
         </is>
@@ -7212,10 +7179,10 @@
           <t>Top 25 Airfields</t>
         </is>
       </c>
-      <c r="E8" s="35" t="n">
+      <c r="E8" s="36" t="n">
         <v>0.4503</v>
       </c>
-      <c r="F8" s="30" t="inlineStr">
+      <c r="F8" s="31" t="inlineStr">
         <is>
           <t>20.28%</t>
         </is>
@@ -7255,10 +7222,10 @@
           <t>Top 25 Airfields</t>
         </is>
       </c>
-      <c r="E9" s="35" t="n">
+      <c r="E9" s="36" t="n">
         <v>0.2867</v>
       </c>
-      <c r="F9" s="30" t="inlineStr">
+      <c r="F9" s="31" t="inlineStr">
         <is>
           <t>8.22%</t>
         </is>
@@ -7266,7 +7233,7 @@
       <c r="G9" s="29" t="n">
         <v>1.44</v>
       </c>
-      <c r="H9" s="32" t="n">
+      <c r="H9" s="33" t="n">
         <v>0.163</v>
       </c>
       <c r="I9" s="9" t="inlineStr">
@@ -7296,10 +7263,10 @@
           <t>63,925 Airport-Days</t>
         </is>
       </c>
-      <c r="E10" s="35" t="n">
+      <c r="E10" s="36" t="n">
         <v>0.4971</v>
       </c>
-      <c r="F10" s="30" t="inlineStr">
+      <c r="F10" s="31" t="inlineStr">
         <is>
           <t>24.71%</t>
         </is>
@@ -7339,10 +7306,10 @@
           <t>Top 25 Airfields</t>
         </is>
       </c>
-      <c r="E11" s="35" t="n">
+      <c r="E11" s="36" t="n">
         <v>0.2019</v>
       </c>
-      <c r="F11" s="30" t="inlineStr">
+      <c r="F11" s="31" t="inlineStr">
         <is>
           <t>4.08%</t>
         </is>
@@ -7350,7 +7317,7 @@
       <c r="G11" s="29" t="n">
         <v>0.99</v>
       </c>
-      <c r="H11" s="32" t="n">
+      <c r="H11" s="33" t="n">
         <v>0.332</v>
       </c>
       <c r="I11" s="9" t="inlineStr">
@@ -7380,10 +7347,10 @@
           <t>Top 25 Airfields</t>
         </is>
       </c>
-      <c r="E12" s="35" t="n">
+      <c r="E12" s="36" t="n">
         <v>0.4375</v>
       </c>
-      <c r="F12" s="30" t="inlineStr">
+      <c r="F12" s="31" t="inlineStr">
         <is>
           <t>19.14%</t>
         </is>
@@ -7423,10 +7390,10 @@
           <t>Top 25 Airfields</t>
         </is>
       </c>
-      <c r="E13" s="35" t="n">
+      <c r="E13" s="36" t="n">
         <v>0.3714</v>
       </c>
-      <c r="F13" s="30" t="inlineStr">
+      <c r="F13" s="31" t="inlineStr">
         <is>
           <t>13.79%</t>
         </is>
@@ -7434,7 +7401,7 @@
       <c r="G13" s="29" t="n">
         <v>1.92</v>
       </c>
-      <c r="H13" s="32" t="n">
+      <c r="H13" s="33" t="n">
         <v>0.067</v>
       </c>
       <c r="I13" s="9" t="inlineStr">
@@ -7464,10 +7431,10 @@
           <t>Top 25 Airfields</t>
         </is>
       </c>
-      <c r="E14" s="35" t="n">
+      <c r="E14" s="36" t="n">
         <v>0.348</v>
       </c>
-      <c r="F14" s="30" t="inlineStr">
+      <c r="F14" s="31" t="inlineStr">
         <is>
           <t>12.11%</t>
         </is>
@@ -7475,7 +7442,7 @@
       <c r="G14" s="29" t="n">
         <v>1.78</v>
       </c>
-      <c r="H14" s="32" t="n">
+      <c r="H14" s="33" t="n">
         <v>0.08799999999999999</v>
       </c>
       <c r="I14" s="9" t="inlineStr">
@@ -7505,10 +7472,10 @@
           <t>7 Days (N=7)</t>
         </is>
       </c>
-      <c r="E15" s="35" t="n">
+      <c r="E15" s="36" t="n">
         <v>0.9022</v>
       </c>
-      <c r="F15" s="30" t="inlineStr">
+      <c r="F15" s="31" t="inlineStr">
         <is>
           <t>81.40%</t>
         </is>
@@ -7548,10 +7515,10 @@
           <t>7 Days (N=7)</t>
         </is>
       </c>
-      <c r="E16" s="35" t="n">
+      <c r="E16" s="36" t="n">
         <v>0.9</v>
       </c>
-      <c r="F16" s="30" t="inlineStr">
+      <c r="F16" s="31" t="inlineStr">
         <is>
           <t>81.00%</t>
         </is>
@@ -7591,15 +7558,15 @@
           <t>12 Months (N=12)</t>
         </is>
       </c>
-      <c r="E17" s="36" t="n">
+      <c r="E17" s="37" t="n">
         <v>0.6313</v>
       </c>
-      <c r="F17" s="31" t="inlineStr">
+      <c r="F17" s="32" t="inlineStr">
         <is>
           <t>39.85%</t>
         </is>
       </c>
-      <c r="G17" s="34" t="n">
+      <c r="G17" s="35" t="n">
         <v>2.57</v>
       </c>
       <c r="H17" s="13" t="inlineStr">

</xml_diff>

<commit_message>
refactor(tables): harmonize Table 4.5 sample grain and synchronize master thesis_tables.xlsx mirrors
</commit_message>
<xml_diff>
--- a/results/manuscript_tables/thesis_tables.xlsx
+++ b/results/manuscript_tables/thesis_tables.xlsx
@@ -6995,7 +6995,7 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="41" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
@@ -7260,7 +7260,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>63,925 Airport-Days</t>
+          <t>Top 25 Airfields</t>
         </is>
       </c>
       <c r="E10" s="36" t="n">

</xml_diff>